<commit_message>
chore(aps): update APS default parameters
- Adjust VALYSAR, THERYS and VOLON residual range and azimuth defaults
- Sync values across global_master_config.yml and facies_aps.dist
- Update ERT design input spreadsheets
- Delete unused fmuconfig/input/aps.yaml
</commit_message>
<xml_diff>
--- a/ert/input/distributions/design_input_ahm.xlsx
+++ b/ert/input/distributions/design_input_ahm.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="general_input" sheetId="1" state="visible" r:id="rId2"/>
@@ -1357,9 +1357,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>153360</xdr:colOff>
+      <xdr:colOff>152640</xdr:colOff>
       <xdr:row>41</xdr:row>
-      <xdr:rowOff>113760</xdr:rowOff>
+      <xdr:rowOff>113040</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1369,7 +1369,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="8130600" cy="7603920"/>
+          <a:ext cx="8148960" cy="7603200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1402,9 +1402,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>153360</xdr:colOff>
+      <xdr:colOff>152640</xdr:colOff>
       <xdr:row>41</xdr:row>
-      <xdr:rowOff>113760</xdr:rowOff>
+      <xdr:rowOff>113040</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1414,7 +1414,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="8130600" cy="7603920"/>
+          <a:ext cx="8148960" cy="7603200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1447,9 +1447,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>153360</xdr:colOff>
+      <xdr:colOff>152640</xdr:colOff>
       <xdr:row>41</xdr:row>
-      <xdr:rowOff>113760</xdr:rowOff>
+      <xdr:rowOff>113040</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1459,7 +1459,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="8130600" cy="7603920"/>
+          <a:ext cx="8148960" cy="7603200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1497,9 +1497,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4292640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1509,7 +1509,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6931440" cy="883440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1542,9 +1542,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4292640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1554,7 +1554,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6931440" cy="883440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1587,9 +1587,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4292640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1599,7 +1599,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6931440" cy="883440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1632,9 +1632,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4292640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1644,7 +1644,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6931440" cy="883440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1677,9 +1677,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4292640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1689,7 +1689,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6931440" cy="883440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1722,9 +1722,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4292640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1734,7 +1734,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6931440" cy="883440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1767,9 +1767,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4292640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1779,7 +1779,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6931440" cy="883440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1812,9 +1812,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4292640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1824,7 +1824,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6931440" cy="883440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1857,9 +1857,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4292640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1869,7 +1869,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6931440" cy="883440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1902,9 +1902,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4292640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1914,7 +1914,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6931440" cy="883440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1947,9 +1947,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4292640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>7200</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1959,7 +1959,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6931440" cy="883440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1992,7 +1992,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.72265625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.13"/>
@@ -2057,7 +2057,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q38"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.72265625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8.44"/>
@@ -2756,7 +2756,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B72"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.72265625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.22"/>
@@ -2855,7 +2855,7 @@
         <v>39</v>
       </c>
       <c r="B12" s="23" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2863,7 +2863,7 @@
         <v>40</v>
       </c>
       <c r="B13" s="23" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2871,7 +2871,7 @@
         <v>41</v>
       </c>
       <c r="B14" s="22" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2879,7 +2879,7 @@
         <v>42</v>
       </c>
       <c r="B15" s="22" t="n">
-        <v>6000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2895,7 +2895,7 @@
         <v>44</v>
       </c>
       <c r="B17" s="22" t="n">
-        <v>300</v>
+        <v>280</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2959,7 +2959,7 @@
         <v>52</v>
       </c>
       <c r="B25" s="22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3031,7 +3031,7 @@
         <v>61</v>
       </c>
       <c r="B34" s="22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3063,7 +3063,7 @@
         <v>65</v>
       </c>
       <c r="B38" s="22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -3117,7 +3117,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AF1048576"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.72265625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58.81"/>
   </cols>
@@ -4496,7 +4496,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.72265625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">

</xml_diff>

<commit_message>
chore(aps): update APS input parameters (#142)
Disable FMU updating of GRF2 for Therys and Volon. Re. Disable FMU updates for Therys and Volon GRF2 #148
Update APS input parameter values
Sync values across global_master_config.yml, facies_aps.dist and ERT design input spreadsheets
Delete unused fmuconfig/input/aps.yaml
Rerun fmudesign to update design matrix output files
</commit_message>
<xml_diff>
--- a/ert/input/distributions/design_input_ahm.xlsx
+++ b/ert/input/distributions/design_input_ahm.xlsx
@@ -731,7 +731,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="71">
   <si>
     <t xml:space="preserve">designtype</t>
   </si>
@@ -871,18 +871,6 @@
     <t xml:space="preserve">THERYS_APS_1_0_GF_GRF1_TREND_STACKANGLE</t>
   </si>
   <si>
-    <t xml:space="preserve">THERYS_APS_1_0_GF_GRF2_RESIDUAL_MAINRANGE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">THERYS_APS_1_0_GF_GRF2_RESIDUAL_PERPRANGE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">THERYS_APS_1_0_GF_GRF2_RESIDUAL_VERTRANGE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">THERYS_APS_1_0_GF_GRF2_RESIDUAL_AZIMUTHANGLE</t>
-  </si>
-  <si>
     <t xml:space="preserve">THERYS_APS_1_0_GF_GRF3_RESIDUAL_MAINRANGE</t>
   </si>
   <si>
@@ -905,18 +893,6 @@
   </si>
   <si>
     <t xml:space="preserve">VOLON_APS_1_0_GF_GRF1_RESIDUAL_AZIMUTHANGLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VOLON_APS_1_0_GF_GRF2_RESIDUAL_MAINRANGE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VOLON_APS_1_0_GF_GRF2_RESIDUAL_PERPRANGE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VOLON_APS_1_0_GF_GRF2_RESIDUAL_VERTRANGE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VOLON_APS_1_0_GF_GRF2_RESIDUAL_AZIMUTHANGLE</t>
   </si>
   <si>
     <t xml:space="preserve">VOLON_APS_1_0_GF_GRF3_RESIDUAL_MAINRANGE</t>
@@ -1357,9 +1333,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>153360</xdr:colOff>
+      <xdr:colOff>151560</xdr:colOff>
       <xdr:row>41</xdr:row>
-      <xdr:rowOff>113760</xdr:rowOff>
+      <xdr:rowOff>111960</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1369,7 +1345,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="8130600" cy="7603920"/>
+          <a:ext cx="8166960" cy="7602120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1402,9 +1378,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>153360</xdr:colOff>
+      <xdr:colOff>151560</xdr:colOff>
       <xdr:row>41</xdr:row>
-      <xdr:rowOff>113760</xdr:rowOff>
+      <xdr:rowOff>111960</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1414,7 +1390,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="8130600" cy="7603920"/>
+          <a:ext cx="8166960" cy="7602120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1447,9 +1423,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>153360</xdr:colOff>
+      <xdr:colOff>151560</xdr:colOff>
       <xdr:row>41</xdr:row>
-      <xdr:rowOff>113760</xdr:rowOff>
+      <xdr:rowOff>111960</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1459,7 +1435,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="8130600" cy="7603920"/>
+          <a:ext cx="8166960" cy="7602120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1497,9 +1473,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4291560</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1509,7 +1485,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6930360" cy="882360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1542,9 +1518,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4291560</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1554,7 +1530,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6930360" cy="882360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1587,9 +1563,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4291560</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1599,7 +1575,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6930360" cy="882360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1632,9 +1608,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4291560</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1644,7 +1620,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6930360" cy="882360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1677,9 +1653,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4291560</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1689,7 +1665,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6930360" cy="882360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1722,9 +1698,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4291560</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1734,7 +1710,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6930360" cy="882360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1767,9 +1743,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4291560</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1779,7 +1755,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6930360" cy="882360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1812,9 +1788,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4291560</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1824,7 +1800,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6930360" cy="882360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1857,9 +1833,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4291560</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1869,7 +1845,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6930360" cy="882360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1902,9 +1878,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4291560</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1914,7 +1890,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6930360" cy="882360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1947,9 +1923,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4293360</xdr:colOff>
+      <xdr:colOff>4291560</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>7920</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1959,7 +1935,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="6932160" cy="884160"/>
+          <a:ext cx="6930360" cy="882360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1992,7 +1968,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.13"/>
@@ -2056,8 +2032,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q38"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:Q1048576"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8.44"/>
@@ -2310,10 +2286,10 @@
         <v>28</v>
       </c>
       <c r="J12" s="19" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K12" s="20" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="O12" s="8" t="s">
         <v>29</v>
@@ -2327,10 +2303,10 @@
         <v>28</v>
       </c>
       <c r="J13" s="19" t="n">
-        <v>7</v>
+        <v>-5</v>
       </c>
       <c r="K13" s="20" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2420,10 +2396,10 @@
         <v>28</v>
       </c>
       <c r="J19" s="19" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="K19" s="20" t="n">
-        <v>8000</v>
+        <v>2000</v>
       </c>
       <c r="O19" s="8" t="s">
         <v>29</v>
@@ -2436,11 +2412,11 @@
       <c r="I20" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="J20" s="7" t="n">
-        <v>750</v>
-      </c>
-      <c r="K20" s="5" t="n">
-        <v>1250</v>
+      <c r="J20" s="19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="K20" s="20" t="n">
+        <v>2000</v>
       </c>
       <c r="O20" s="8" t="s">
         <v>29</v>
@@ -2454,10 +2430,10 @@
         <v>28</v>
       </c>
       <c r="J21" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="20" t="n">
         <v>3</v>
-      </c>
-      <c r="K21" s="20" t="n">
-        <v>7</v>
       </c>
       <c r="O21" s="8" t="s">
         <v>29</v>
@@ -2485,10 +2461,10 @@
         <v>28</v>
       </c>
       <c r="J23" s="19" t="n">
-        <v>1000</v>
+        <v>550</v>
       </c>
       <c r="K23" s="20" t="n">
-        <v>2000</v>
+        <v>1275</v>
       </c>
       <c r="O23" s="8" t="s">
         <v>29</v>
@@ -2502,10 +2478,10 @@
         <v>28</v>
       </c>
       <c r="J24" s="19" t="n">
-        <v>1000</v>
+        <v>120</v>
       </c>
       <c r="K24" s="20" t="n">
-        <v>2000</v>
+        <v>275</v>
       </c>
       <c r="O24" s="8" t="s">
         <v>29</v>
@@ -2519,10 +2495,10 @@
         <v>28</v>
       </c>
       <c r="J25" s="19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K25" s="20" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="O25" s="8" t="s">
         <v>29</v>
@@ -2536,10 +2512,10 @@
         <v>28</v>
       </c>
       <c r="J26" s="19" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K26" s="20" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2550,10 +2526,10 @@
         <v>28</v>
       </c>
       <c r="J27" s="19" t="n">
-        <v>550</v>
+        <v>475</v>
       </c>
       <c r="K27" s="20" t="n">
-        <v>1275</v>
+        <v>1150</v>
       </c>
       <c r="O27" s="8" t="s">
         <v>29</v>
@@ -2567,10 +2543,10 @@
         <v>28</v>
       </c>
       <c r="J28" s="19" t="n">
-        <v>120</v>
+        <v>475</v>
       </c>
       <c r="K28" s="20" t="n">
-        <v>275</v>
+        <v>1150</v>
       </c>
       <c r="O28" s="8" t="s">
         <v>29</v>
@@ -2584,10 +2560,10 @@
         <v>28</v>
       </c>
       <c r="J29" s="19" t="n">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="K29" s="20" t="n">
-        <v>7</v>
+        <v>1.5</v>
       </c>
       <c r="O29" s="8" t="s">
         <v>29</v>
@@ -2601,142 +2577,20 @@
         <v>28</v>
       </c>
       <c r="J30" s="19" t="n">
-        <v>3</v>
+        <v>-5</v>
       </c>
       <c r="K30" s="20" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D31" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="I31" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J31" s="7" t="n">
-        <v>550</v>
-      </c>
-      <c r="K31" s="5" t="n">
-        <v>1425</v>
-      </c>
-      <c r="O31" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D32" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="I32" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J32" s="7" t="n">
-        <v>550</v>
-      </c>
-      <c r="K32" s="5" t="n">
-        <v>1425</v>
-      </c>
-      <c r="O32" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D33" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="I33" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J33" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="K33" s="20" t="n">
-        <v>7</v>
-      </c>
-      <c r="O33" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D34" s="0" t="s">
-        <v>61</v>
-      </c>
-      <c r="I34" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J34" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="K34" s="20" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D35" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="I35" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J35" s="19" t="n">
-        <v>475</v>
-      </c>
-      <c r="K35" s="20" t="n">
-        <v>1150</v>
-      </c>
-      <c r="O35" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D36" s="0" t="s">
-        <v>63</v>
-      </c>
-      <c r="I36" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J36" s="19" t="n">
-        <v>475</v>
-      </c>
-      <c r="K36" s="20" t="n">
-        <v>1150</v>
-      </c>
-      <c r="O36" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D37" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="I37" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J37" s="19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K37" s="20" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="O37" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D38" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="I38" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J38" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="K38" s="20" t="n">
-        <v>7</v>
-      </c>
-    </row>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -2755,8 +2609,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B72"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B1048576"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60.87"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14.22"/>
@@ -2767,7 +2621,7 @@
         <v>11</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2855,7 +2709,7 @@
         <v>39</v>
       </c>
       <c r="B12" s="23" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2871,7 +2725,7 @@
         <v>41</v>
       </c>
       <c r="B14" s="22" t="n">
-        <v>1000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2879,7 +2733,7 @@
         <v>42</v>
       </c>
       <c r="B15" s="22" t="n">
-        <v>6000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2895,7 +2749,7 @@
         <v>44</v>
       </c>
       <c r="B17" s="22" t="n">
-        <v>300</v>
+        <v>280</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2911,7 +2765,7 @@
         <v>46</v>
       </c>
       <c r="B19" s="22" t="n">
-        <v>6000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2919,7 +2773,7 @@
         <v>47</v>
       </c>
       <c r="B20" s="22" t="n">
-        <v>1000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2927,7 +2781,7 @@
         <v>48</v>
       </c>
       <c r="B21" s="22" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2943,7 +2797,7 @@
         <v>50</v>
       </c>
       <c r="B23" s="22" t="n">
-        <v>1500</v>
+        <v>900</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2951,7 +2805,7 @@
         <v>51</v>
       </c>
       <c r="B24" s="22" t="n">
-        <v>1500</v>
+        <v>200</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2959,7 +2813,7 @@
         <v>52</v>
       </c>
       <c r="B25" s="22" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2967,7 +2821,7 @@
         <v>53</v>
       </c>
       <c r="B26" s="22" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2975,7 +2829,7 @@
         <v>54</v>
       </c>
       <c r="B27" s="22" t="n">
-        <v>900</v>
+        <v>800</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2983,7 +2837,7 @@
         <v>55</v>
       </c>
       <c r="B28" s="22" t="n">
-        <v>200</v>
+        <v>800</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2991,7 +2845,7 @@
         <v>56</v>
       </c>
       <c r="B29" s="22" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2999,73 +2853,17 @@
         <v>57</v>
       </c>
       <c r="B30" s="22" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="B31" s="22" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="B32" s="22" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="B33" s="22" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
-        <v>61</v>
-      </c>
-      <c r="B34" s="22" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="B35" s="22" t="n">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
-        <v>63</v>
-      </c>
-      <c r="B36" s="22" t="n">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="B37" s="22" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
-        <v>65</v>
-      </c>
-      <c r="B38" s="22" t="n">
-        <v>0</v>
-      </c>
-    </row>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -3092,14 +2890,14 @@
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -3116,10 +2914,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AF1048576"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:Z22"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1019" style="0" width="11.52"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="246.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3186,28 +2985,10 @@
       <c r="V1" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="W1" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="X1" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y1" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z1" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="AA1" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="AB1" s="24" t="s">
-        <v>64</v>
-      </c>
-      <c r="AC1" s="25"/>
-      <c r="AD1" s="25"/>
-      <c r="AE1" s="25"/>
-      <c r="AF1" s="25"/>
+      <c r="W1" s="25"/>
+      <c r="X1" s="25"/>
+      <c r="Y1" s="25"/>
+      <c r="Z1" s="25"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
@@ -3676,22 +3457,22 @@
         <v>0</v>
       </c>
       <c r="K17" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="L17" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="M17" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="N17" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="O17" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="P17" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="0" t="n">
         <v>1</v>
@@ -3729,22 +3510,22 @@
         <v>0</v>
       </c>
       <c r="K18" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="L18" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="M18" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="N18" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="O18" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="P18" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="0" t="n">
         <v>0.9</v>
@@ -3785,22 +3566,22 @@
         <v>0</v>
       </c>
       <c r="K19" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="L19" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="M19" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="N19" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="O19" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="P19" s="0" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="0" t="n">
         <v>0.9</v>
@@ -3862,13 +3643,13 @@
         <v>0</v>
       </c>
       <c r="Q20" s="0" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="R20" s="0" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="S20" s="0" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="T20" s="0" t="n">
         <v>1</v>
@@ -3924,13 +3705,13 @@
         <v>0</v>
       </c>
       <c r="Q21" s="0" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="R21" s="0" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="S21" s="0" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="T21" s="0" t="n">
         <v>0.9</v>
@@ -3989,13 +3770,13 @@
         <v>0</v>
       </c>
       <c r="Q22" s="0" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="R22" s="0" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="S22" s="0" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="T22" s="0" t="n">
         <v>0.9</v>
@@ -4007,478 +3788,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
-        <v>58</v>
-      </c>
-      <c r="B23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="S23" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="T23" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="U23" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="V23" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="W23" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="B24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="S24" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="T24" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="U24" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="V24" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="W24" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="X24" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="B25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="S25" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="T25" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="U25" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="V25" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="W25" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="X25" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="Y25" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="B26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="S26" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="T26" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="U26" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="V26" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="W26" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="X26" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="Y26" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="Z26" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
-        <v>63</v>
-      </c>
-      <c r="B27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="S27" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="T27" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="U27" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="V27" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="W27" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="X27" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="Y27" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="Z27" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="AA27" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="B28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="S28" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="U28" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="V28" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="W28" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="X28" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="Y28" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="Z28" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="AA28" s="0" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="AB28" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -4496,58 +3805,58 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D9" s="26" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>